<commit_message>
added parts for ashlynn
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5F6B6F-6E3B-4E75-9446-CFB734BE530D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FB77531-BB17-43DB-8EB8-BF3D267EFD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" firstSheet="1" activeTab="2" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="11170" firstSheet="1" activeTab="6" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1494" uniqueCount="872">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1527" uniqueCount="892">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1669,30 +1669,9 @@
     <t>3.48 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
   </si>
   <si>
-    <t>SPI-CAN Bridge</t>
-  </si>
-  <si>
-    <t>MCP2518FDT-E/SL</t>
-  </si>
-  <si>
     <t>Uses single-ended CAN</t>
   </si>
   <si>
-    <t>CAN Controller CAN 2.0 SPI Interface 14-SOIC</t>
-  </si>
-  <si>
-    <t>CAN Frontend Transceiver</t>
-  </si>
-  <si>
-    <t>Single-ended CAN to CAN FD</t>
-  </si>
-  <si>
-    <t>ATA6561-GAQW-N</t>
-  </si>
-  <si>
-    <t>1/1 Transceiver CANbus 8-SO</t>
-  </si>
-  <si>
     <t>RC0603FR-07120RL</t>
   </si>
   <si>
@@ -2675,6 +2654,87 @@
   </si>
   <si>
     <t>Aluminum Unthreaded Spacer</t>
+  </si>
+  <si>
+    <t>Pogo</t>
+  </si>
+  <si>
+    <t>5358</t>
+  </si>
+  <si>
+    <t>Magnetic Right-Angle Thru-Hole</t>
+  </si>
+  <si>
+    <t>4 Position Spring Piston Connector Panel Mount; Through Hole, Right Angle</t>
+  </si>
+  <si>
+    <t>6.8uH</t>
+  </si>
+  <si>
+    <t>6.9A</t>
+  </si>
+  <si>
+    <t>SMD 8.50 x 8.00mm</t>
+  </si>
+  <si>
+    <t>6.8 µH Shielded Drum Core, Wirewound Inductor 6.9 A 25.85mOhm Max 2-SMD, J-Lead</t>
+  </si>
+  <si>
+    <t>ETQ-P4M6R8KVK</t>
+  </si>
+  <si>
+    <t>158k</t>
+  </si>
+  <si>
+    <t>RC0603FR-07158KL</t>
+  </si>
+  <si>
+    <t>158 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
+  </si>
+  <si>
+    <t>MCP2515T-I/SO</t>
+  </si>
+  <si>
+    <t>CANbus Controller CAN 2.0 SPI Interface 18-SOIC</t>
+  </si>
+  <si>
+    <t>CAN-SPI Bridge</t>
+  </si>
+  <si>
+    <t>TJA1050T/CM,118</t>
+  </si>
+  <si>
+    <t>1/1 Transceiver Half CANbus 8-SO</t>
+  </si>
+  <si>
+    <t>CAN FD Front End</t>
+  </si>
+  <si>
+    <t>8MHz</t>
+  </si>
+  <si>
+    <t>18pF</t>
+  </si>
+  <si>
+    <t>ABM3-8.000MHZ-D2Y-T</t>
+  </si>
+  <si>
+    <t>8 MHz ±20ppm Crystal 18pF 140 Ohms 2-SMD, No Lead</t>
+  </si>
+  <si>
+    <t>WCS1600</t>
+  </si>
+  <si>
+    <t>Series / Purpose</t>
+  </si>
+  <si>
+    <t>Current Monitor</t>
+  </si>
+  <si>
+    <t>Hall Effect</t>
+  </si>
+  <si>
+    <t>https://www.winson.com.tw/uploads/images/WCS1600.pdf</t>
   </si>
 </sst>
 </file>
@@ -2857,6 +2917,57 @@
           <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -3126,57 +3237,6 @@
         </ext>
       </extLst>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3221,13 +3281,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I49" totalsRowShown="0">
   <autoFilter ref="A1:I49" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="78"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="77"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="76"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="75"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -3239,11 +3299,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H20" totalsRowShown="0">
   <autoFilter ref="A1:H20" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="42"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="41"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="40"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -3253,10 +3313,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="39">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="38"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -3275,7 +3335,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="37"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -3285,54 +3345,54 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="36">
   <autoFilter ref="A1:H11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="8">
-    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="24"/>
-    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="15"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="19"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:H100" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="C1:C50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="76"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="74">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="11">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -3340,11 +3400,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="73"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3422,20 +3482,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="74">
   <autoFilter ref="A1:H100" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H100">
     <sortCondition ref="B1:B100"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="63"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="62"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="61"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="60"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="59"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="58"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="57"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="56"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="73"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="72"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="71"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="70"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="69"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="68"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="67"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="66"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3458,13 +3518,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="65">
   <autoFilter ref="A1:H20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H20">
     <sortCondition ref="B1:B20"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="64"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -3484,8 +3544,8 @@
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="53"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="63"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="62"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -3495,11 +3555,11 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="51">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="61">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="50"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="60"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series / Purpose" dataDxfId="59"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -3510,25 +3570,25 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="58">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="47"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="52">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="41"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="50"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -3542,15 +3602,15 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:F11" totalsRowShown="0" headerRowDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:F11" totalsRowShown="0" headerRowDxfId="49">
   <autoFilter ref="A1:F11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="6">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="38"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{B8135C27-240F-4D83-9F04-23BE8CE5150A}" name="Max Current" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="48"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{B8135C27-240F-4D83-9F04-23BE8CE5150A}" name="Max Current" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4006,7 +4066,7 @@
         <v>46</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>858</v>
+        <v>851</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>213</v>
@@ -4057,16 +4117,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>662</v>
+        <v>655</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>664</v>
+        <v>657</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>665</v>
+        <v>658</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -4080,10 +4140,10 @@
         <v>213</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>692</v>
+        <v>685</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>693</v>
+        <v>686</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -4094,21 +4154,36 @@
         <v>46</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>854</v>
+        <v>847</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>857</v>
+        <v>850</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>855</v>
+        <v>848</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>856</v>
+        <v>849</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>869</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>870</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>871</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>873</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>872</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -4390,7 +4465,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>598</v>
+        <v>591</v>
       </c>
       <c r="C11" t="s">
         <v>361</v>
@@ -4399,16 +4474,16 @@
         <v>103</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>599</v>
+        <v>592</v>
       </c>
       <c r="F11" t="s">
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>600</v>
+        <v>593</v>
       </c>
       <c r="H11" t="s">
-        <v>601</v>
+        <v>594</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -4416,7 +4491,7 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>715</v>
+        <v>708</v>
       </c>
       <c r="C12" t="s">
         <v>415</v>
@@ -4425,16 +4500,16 @@
         <v>103</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>716</v>
+        <v>709</v>
       </c>
       <c r="F12" t="s">
         <v>360</v>
       </c>
       <c r="G12" t="s">
-        <v>717</v>
+        <v>710</v>
       </c>
       <c r="H12" t="s">
-        <v>718</v>
+        <v>711</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -4728,10 +4803,10 @@
         <v>232</v>
       </c>
       <c r="C8" t="s">
-        <v>588</v>
+        <v>581</v>
       </c>
       <c r="D8" t="s">
-        <v>589</v>
+        <v>582</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -4742,10 +4817,10 @@
         <v>232</v>
       </c>
       <c r="C9" t="s">
-        <v>595</v>
+        <v>588</v>
       </c>
       <c r="D9" t="s">
-        <v>596</v>
+        <v>589</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -5244,10 +5319,10 @@
         <v>193</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>544</v>
+        <v>537</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>545</v>
+        <v>538</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -5271,10 +5346,10 @@
         <v>137</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>606</v>
+        <v>599</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>607</v>
+        <v>600</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -5903,7 +5978,7 @@
         <v>1</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>568</v>
+        <v>561</v>
       </c>
       <c r="C31" s="17">
         <f t="shared" si="0"/>
@@ -5919,10 +5994,10 @@
         <v>193</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>569</v>
+        <v>562</v>
       </c>
       <c r="H31" s="16" t="s">
-        <v>570</v>
+        <v>563</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -5946,10 +6021,10 @@
         <v>193</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>571</v>
+        <v>564</v>
       </c>
       <c r="H32" s="16" t="s">
-        <v>572</v>
+        <v>565</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
@@ -5973,10 +6048,10 @@
         <v>193</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>573</v>
+        <v>566</v>
       </c>
       <c r="H33" s="16" t="s">
-        <v>574</v>
+        <v>567</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
@@ -5984,7 +6059,7 @@
         <v>1</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>578</v>
+        <v>571</v>
       </c>
       <c r="C34" s="17">
         <f t="shared" ref="C34:C97" si="1">IF(ISNUMBER(B34),
@@ -6005,10 +6080,10 @@
         <v>193</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>579</v>
+        <v>572</v>
       </c>
       <c r="H34" s="16" t="s">
-        <v>580</v>
+        <v>573</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
@@ -6026,16 +6101,16 @@
         <v>62</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>620</v>
+        <v>613</v>
       </c>
       <c r="F35" s="16" t="s">
-        <v>617</v>
+        <v>610</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>621</v>
+        <v>614</v>
       </c>
       <c r="H35" s="16" t="s">
-        <v>622</v>
+        <v>615</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
@@ -6050,7 +6125,7 @@
         <v>10</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>700</v>
+        <v>693</v>
       </c>
       <c r="E36" s="16" t="s">
         <v>8</v>
@@ -6059,10 +6134,10 @@
         <v>193</v>
       </c>
       <c r="G36" s="16" t="s">
-        <v>701</v>
+        <v>694</v>
       </c>
       <c r="H36" s="16" t="s">
-        <v>702</v>
+        <v>695</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
@@ -6070,7 +6145,7 @@
         <v>1</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>780</v>
+        <v>773</v>
       </c>
       <c r="C37" s="17">
         <f t="shared" si="1"/>
@@ -6086,10 +6161,10 @@
         <v>193</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>779</v>
+        <v>772</v>
       </c>
       <c r="H37" s="16" t="s">
-        <v>781</v>
+        <v>774</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
@@ -6097,7 +6172,7 @@
         <v>1</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>783</v>
+        <v>776</v>
       </c>
       <c r="C38" s="17">
         <f t="shared" si="1"/>
@@ -6113,10 +6188,10 @@
         <v>193</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="H38" s="16" t="s">
-        <v>784</v>
+        <v>777</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
@@ -6124,7 +6199,7 @@
         <v>1</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>785</v>
+        <v>778</v>
       </c>
       <c r="C39" s="17">
         <f t="shared" si="1"/>
@@ -6140,10 +6215,10 @@
         <v>193</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>786</v>
+        <v>779</v>
       </c>
       <c r="H39" s="16" t="s">
-        <v>787</v>
+        <v>780</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
@@ -6151,7 +6226,7 @@
         <v>1</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>788</v>
+        <v>781</v>
       </c>
       <c r="C40" s="17">
         <f t="shared" si="1"/>
@@ -6167,10 +6242,10 @@
         <v>193</v>
       </c>
       <c r="G40" s="16" t="s">
-        <v>789</v>
+        <v>782</v>
       </c>
       <c r="H40" s="16" t="s">
-        <v>790</v>
+        <v>783</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
@@ -6178,7 +6253,7 @@
         <v>1</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>792</v>
+        <v>785</v>
       </c>
       <c r="C41" s="17">
         <f t="shared" si="1"/>
@@ -6194,10 +6269,10 @@
         <v>193</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>791</v>
+        <v>784</v>
       </c>
       <c r="H41" s="16" t="s">
-        <v>793</v>
+        <v>786</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.35">
@@ -6205,7 +6280,7 @@
         <v>1</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>794</v>
+        <v>787</v>
       </c>
       <c r="C42" s="17">
         <f t="shared" si="1"/>
@@ -6221,10 +6296,10 @@
         <v>193</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>795</v>
+        <v>788</v>
       </c>
       <c r="H42" s="16" t="s">
-        <v>796</v>
+        <v>789</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
@@ -6232,7 +6307,7 @@
         <v>1</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>797</v>
+        <v>790</v>
       </c>
       <c r="C43" s="17">
         <f t="shared" si="1"/>
@@ -6248,10 +6323,10 @@
         <v>137</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>798</v>
+        <v>791</v>
       </c>
       <c r="H43" s="16" t="s">
-        <v>799</v>
+        <v>792</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
@@ -6259,7 +6334,7 @@
         <v>1</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="C44" s="17">
         <f t="shared" si="1"/>
@@ -6275,10 +6350,10 @@
         <v>193</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>801</v>
+        <v>794</v>
       </c>
       <c r="H44" s="16" t="s">
-        <v>802</v>
+        <v>795</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
@@ -6286,7 +6361,7 @@
         <v>1</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>803</v>
+        <v>796</v>
       </c>
       <c r="C45" s="17">
         <f t="shared" si="1"/>
@@ -6302,10 +6377,10 @@
         <v>193</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>804</v>
+        <v>797</v>
       </c>
       <c r="H45" s="16" t="s">
-        <v>805</v>
+        <v>798</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
@@ -6313,7 +6388,7 @@
         <v>1</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>807</v>
+        <v>800</v>
       </c>
       <c r="C46" s="17">
         <f t="shared" si="1"/>
@@ -6329,10 +6404,10 @@
         <v>193</v>
       </c>
       <c r="G46" s="16" t="s">
-        <v>806</v>
+        <v>799</v>
       </c>
       <c r="H46" s="16" t="s">
-        <v>808</v>
+        <v>801</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
@@ -6340,7 +6415,7 @@
         <v>1</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>859</v>
+        <v>852</v>
       </c>
       <c r="C47" s="17">
         <f t="shared" si="1"/>
@@ -6356,10 +6431,10 @@
         <v>193</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>860</v>
+        <v>853</v>
       </c>
       <c r="H47" s="16" t="s">
-        <v>861</v>
+        <v>854</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
@@ -6367,7 +6442,7 @@
         <v>1</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>862</v>
+        <v>855</v>
       </c>
       <c r="C48" s="17">
         <f t="shared" si="1"/>
@@ -6383,28 +6458,38 @@
         <v>193</v>
       </c>
       <c r="G48" s="16" t="s">
-        <v>863</v>
+        <v>856</v>
       </c>
       <c r="H48" s="16" t="s">
-        <v>864</v>
+        <v>857</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B49" s="15">
-        <v>0</v>
-      </c>
-      <c r="C49" s="17" t="str">
+        <v>1</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>874</v>
+      </c>
+      <c r="C49" s="17">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="D49" s="16"/>
-      <c r="E49" s="16"/>
-      <c r="F49" s="16"/>
-      <c r="G49" s="16"/>
-      <c r="H49" s="16"/>
+        <v>158000</v>
+      </c>
+      <c r="D49" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="E49" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="G49" s="16" t="s">
+        <v>875</v>
+      </c>
+      <c r="H49" s="16" t="s">
+        <v>876</v>
+      </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="18" t="b">
@@ -7415,22 +7500,22 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>602</v>
+        <v>595</v>
       </c>
       <c r="C6" t="s">
         <v>72</v>
       </c>
       <c r="D6" t="s">
-        <v>603</v>
+        <v>596</v>
       </c>
       <c r="E6" t="s">
         <v>74</v>
       </c>
       <c r="F6" t="s">
-        <v>604</v>
+        <v>597</v>
       </c>
       <c r="G6" t="s">
-        <v>605</v>
+        <v>598</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -7438,22 +7523,22 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>833</v>
+        <v>826</v>
       </c>
       <c r="C7" t="s">
         <v>310</v>
       </c>
       <c r="D7" t="s">
-        <v>834</v>
+        <v>827</v>
       </c>
       <c r="E7" t="s">
         <v>171</v>
       </c>
       <c r="F7" t="s">
-        <v>835</v>
+        <v>828</v>
       </c>
       <c r="G7" t="s">
-        <v>836</v>
+        <v>829</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -7632,13 +7717,13 @@
         <v>295</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>736</v>
+        <v>729</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>739</v>
+        <v>732</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="G1" s="21" t="s">
         <v>297</v>
@@ -7690,19 +7775,19 @@
         <v>117</v>
       </c>
       <c r="E3" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="F3" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="G3" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="H3" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="I3" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -7716,22 +7801,22 @@
         <v>298</v>
       </c>
       <c r="D4" t="s">
-        <v>738</v>
+        <v>731</v>
       </c>
       <c r="E4" t="s">
-        <v>591</v>
+        <v>584</v>
       </c>
       <c r="F4" t="s">
-        <v>592</v>
+        <v>585</v>
       </c>
       <c r="G4" t="s">
-        <v>590</v>
+        <v>583</v>
       </c>
       <c r="H4" t="s">
-        <v>593</v>
+        <v>586</v>
       </c>
       <c r="I4" t="s">
-        <v>594</v>
+        <v>587</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -7739,28 +7824,28 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>695</v>
+        <v>688</v>
       </c>
       <c r="C5" t="s">
-        <v>694</v>
+        <v>687</v>
       </c>
       <c r="D5" t="s">
-        <v>738</v>
+        <v>731</v>
       </c>
       <c r="E5" t="s">
-        <v>740</v>
+        <v>733</v>
       </c>
       <c r="F5" t="s">
-        <v>696</v>
+        <v>689</v>
       </c>
       <c r="G5" t="s">
-        <v>697</v>
+        <v>690</v>
       </c>
       <c r="H5" t="s">
-        <v>699</v>
+        <v>692</v>
       </c>
       <c r="I5" t="s">
-        <v>698</v>
+        <v>691</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -7771,25 +7856,25 @@
         <v>296</v>
       </c>
       <c r="C6" t="s">
+        <v>727</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>730</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>734</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>737</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>741</v>
-      </c>
       <c r="F6" t="s">
-        <v>742</v>
+        <v>735</v>
       </c>
       <c r="G6" t="s">
-        <v>590</v>
+        <v>583</v>
       </c>
       <c r="H6" t="s">
-        <v>735</v>
+        <v>728</v>
       </c>
       <c r="I6" t="s">
-        <v>743</v>
+        <v>736</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -7806,19 +7891,19 @@
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>771</v>
+        <v>764</v>
       </c>
       <c r="F7" t="s">
-        <v>772</v>
+        <v>765</v>
       </c>
       <c r="G7" t="s">
-        <v>773</v>
+        <v>766</v>
       </c>
       <c r="H7" t="s">
-        <v>770</v>
+        <v>763</v>
       </c>
       <c r="I7" t="s">
-        <v>774</v>
+        <v>767</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -7835,19 +7920,19 @@
         <v>106</v>
       </c>
       <c r="E8" t="s">
-        <v>775</v>
+        <v>768</v>
       </c>
       <c r="F8" t="s">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="G8" t="s">
-        <v>820</v>
+        <v>813</v>
       </c>
       <c r="H8" t="s">
-        <v>777</v>
+        <v>770</v>
       </c>
       <c r="I8" t="s">
-        <v>778</v>
+        <v>771</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -7861,22 +7946,22 @@
         <v>298</v>
       </c>
       <c r="D9" t="s">
-        <v>666</v>
+        <v>659</v>
       </c>
       <c r="E9" t="s">
-        <v>818</v>
+        <v>811</v>
       </c>
       <c r="F9" t="s">
-        <v>819</v>
+        <v>812</v>
       </c>
       <c r="G9" t="s">
-        <v>820</v>
+        <v>813</v>
       </c>
       <c r="H9" t="s">
-        <v>821</v>
+        <v>814</v>
       </c>
       <c r="I9" t="s">
-        <v>822</v>
+        <v>815</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -8113,7 +8198,7 @@
         <v>9</v>
       </c>
       <c r="I2" t="s">
-        <v>597</v>
+        <v>590</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -8704,7 +8789,7 @@
         <v>109</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>557</v>
+        <v>550</v>
       </c>
       <c r="D23" t="s">
         <v>343</v>
@@ -8722,7 +8807,7 @@
         <v>112</v>
       </c>
       <c r="I23" t="s">
-        <v>558</v>
+        <v>551</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
@@ -8730,7 +8815,7 @@
         <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>566</v>
+        <v>559</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>23</v>
@@ -8751,7 +8836,7 @@
         <v>9</v>
       </c>
       <c r="I24" t="s">
-        <v>567</v>
+        <v>560</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
@@ -8780,7 +8865,7 @@
         <v>9</v>
       </c>
       <c r="I25" t="s">
-        <v>581</v>
+        <v>574</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
@@ -8788,7 +8873,7 @@
         <v>1</v>
       </c>
       <c r="B26" t="s">
-        <v>627</v>
+        <v>620</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>8</v>
@@ -8809,7 +8894,7 @@
         <v>9</v>
       </c>
       <c r="I26" t="s">
-        <v>628</v>
+        <v>621</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
@@ -8817,10 +8902,10 @@
         <v>1</v>
       </c>
       <c r="B27" t="s">
-        <v>660</v>
+        <v>653</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>557</v>
+        <v>550</v>
       </c>
       <c r="D27" t="s">
         <v>343</v>
@@ -8838,7 +8923,7 @@
         <v>112</v>
       </c>
       <c r="I27" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
@@ -8846,7 +8931,7 @@
         <v>1</v>
       </c>
       <c r="B28" t="s">
-        <v>677</v>
+        <v>670</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>8</v>
@@ -8867,7 +8952,7 @@
         <v>9</v>
       </c>
       <c r="I28" t="s">
-        <v>678</v>
+        <v>671</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
@@ -8896,7 +8981,7 @@
         <v>112</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>769</v>
+        <v>762</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
@@ -8904,7 +8989,7 @@
         <v>1</v>
       </c>
       <c r="B30" t="s">
-        <v>848</v>
+        <v>841</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>8</v>
@@ -8925,7 +9010,7 @@
         <v>9</v>
       </c>
       <c r="I30" t="s">
-        <v>847</v>
+        <v>840</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
@@ -8933,7 +9018,7 @@
         <v>1</v>
       </c>
       <c r="B31" t="s">
-        <v>865</v>
+        <v>858</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>8</v>
@@ -8954,7 +9039,7 @@
         <v>9</v>
       </c>
       <c r="I31" t="s">
-        <v>866</v>
+        <v>859</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
@@ -8965,7 +9050,7 @@
         <v>10</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>620</v>
+        <v>613</v>
       </c>
       <c r="D32" t="s">
         <v>106</v>
@@ -8983,7 +9068,7 @@
         <v>9</v>
       </c>
       <c r="I32" t="s">
-        <v>867</v>
+        <v>860</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
@@ -9176,7 +9261,7 @@
         <v>125</v>
       </c>
       <c r="H3" t="s">
-        <v>814</v>
+        <v>807</v>
       </c>
       <c r="I3" t="s">
         <v>366</v>
@@ -9225,22 +9310,22 @@
         <v>363</v>
       </c>
       <c r="D5" t="s">
-        <v>623</v>
+        <v>616</v>
       </c>
       <c r="E5" t="s">
-        <v>604</v>
+        <v>597</v>
       </c>
       <c r="F5" t="s">
-        <v>624</v>
+        <v>617</v>
       </c>
       <c r="G5" t="s">
         <v>103</v>
       </c>
       <c r="I5" t="s">
-        <v>625</v>
+        <v>618</v>
       </c>
       <c r="J5" t="s">
-        <v>626</v>
+        <v>619</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -9254,22 +9339,22 @@
         <v>363</v>
       </c>
       <c r="D6" t="s">
-        <v>552</v>
+        <v>545</v>
       </c>
       <c r="E6" t="s">
         <v>86</v>
       </c>
       <c r="F6" t="s">
-        <v>729</v>
+        <v>722</v>
       </c>
       <c r="G6" t="s">
         <v>103</v>
       </c>
       <c r="I6" t="s">
-        <v>730</v>
+        <v>723</v>
       </c>
       <c r="J6" t="s">
-        <v>731</v>
+        <v>724</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -9283,7 +9368,7 @@
         <v>363</v>
       </c>
       <c r="D7" t="s">
-        <v>552</v>
+        <v>545</v>
       </c>
       <c r="E7" t="s">
         <v>86</v>
@@ -9295,10 +9380,10 @@
         <v>103</v>
       </c>
       <c r="I7" t="s">
-        <v>732</v>
+        <v>725</v>
       </c>
       <c r="J7" t="s">
-        <v>733</v>
+        <v>726</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -9324,7 +9409,7 @@
         <v>103</v>
       </c>
       <c r="H8" t="s">
-        <v>815</v>
+        <v>808</v>
       </c>
       <c r="I8" t="s">
         <v>145</v>
@@ -9344,10 +9429,10 @@
         <v>224</v>
       </c>
       <c r="D9" t="s">
-        <v>555</v>
+        <v>548</v>
       </c>
       <c r="E9" t="s">
-        <v>552</v>
+        <v>545</v>
       </c>
       <c r="F9" t="s">
         <v>392</v>
@@ -9356,10 +9441,10 @@
         <v>103</v>
       </c>
       <c r="I9" t="s">
-        <v>553</v>
+        <v>546</v>
       </c>
       <c r="J9" t="s">
-        <v>554</v>
+        <v>547</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -9373,10 +9458,10 @@
         <v>224</v>
       </c>
       <c r="D10" t="s">
-        <v>657</v>
+        <v>650</v>
       </c>
       <c r="E10" t="s">
-        <v>604</v>
+        <v>597</v>
       </c>
       <c r="F10" t="s">
         <v>119</v>
@@ -9385,10 +9470,10 @@
         <v>103</v>
       </c>
       <c r="I10" t="s">
-        <v>658</v>
+        <v>651</v>
       </c>
       <c r="J10" t="s">
-        <v>659</v>
+        <v>652</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
@@ -9402,30 +9487,30 @@
         <v>224</v>
       </c>
       <c r="D11" t="s">
-        <v>811</v>
+        <v>804</v>
       </c>
       <c r="E11" t="s">
-        <v>812</v>
+        <v>805</v>
       </c>
       <c r="F11" t="s">
-        <v>810</v>
+        <v>803</v>
       </c>
       <c r="G11" t="s">
         <v>103</v>
       </c>
       <c r="H11" t="s">
-        <v>815</v>
+        <v>808</v>
       </c>
       <c r="I11" t="s">
-        <v>809</v>
+        <v>802</v>
       </c>
       <c r="J11" t="s">
-        <v>813</v>
+        <v>806</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
         <v>143</v>
@@ -9434,10 +9519,10 @@
         <v>224</v>
       </c>
       <c r="D12" t="s">
-        <v>851</v>
+        <v>844</v>
       </c>
       <c r="E12" t="s">
-        <v>852</v>
+        <v>845</v>
       </c>
       <c r="F12" t="s">
         <v>119</v>
@@ -9446,13 +9531,13 @@
         <v>103</v>
       </c>
       <c r="H12" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
       <c r="I12" t="s">
-        <v>849</v>
+        <v>842</v>
       </c>
       <c r="J12" t="s">
-        <v>850</v>
+        <v>843</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -9828,7 +9913,7 @@
         <v>331</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>556</v>
+        <v>549</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -10138,16 +10223,16 @@
         <v>331</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>652</v>
+        <v>645</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>653</v>
+        <v>646</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>654</v>
+        <v>647</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>655</v>
+        <v>648</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
@@ -10155,7 +10240,7 @@
         <v>1</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>640</v>
+        <v>633</v>
       </c>
       <c r="C30" s="12">
         <v>3</v>
@@ -10164,16 +10249,16 @@
         <v>331</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>641</v>
+        <v>634</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>643</v>
+        <v>636</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>642</v>
+        <v>635</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>644</v>
+        <v>637</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
@@ -10181,7 +10266,7 @@
         <v>1</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>640</v>
+        <v>633</v>
       </c>
       <c r="C31" s="12">
         <v>2</v>
@@ -10190,16 +10275,16 @@
         <v>331</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>649</v>
+        <v>642</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>642</v>
+        <v>635</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>651</v>
+        <v>644</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -10207,7 +10292,7 @@
         <v>1</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>656</v>
+        <v>649</v>
       </c>
       <c r="C32" s="12">
         <v>10</v>
@@ -10227,7 +10312,7 @@
         <v>1</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>656</v>
+        <v>649</v>
       </c>
       <c r="C33" s="12">
         <v>16</v>
@@ -10410,13 +10495,13 @@
         <v>331</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>550</v>
+        <v>543</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>410</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>551</v>
+        <v>544</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
@@ -10456,13 +10541,13 @@
         <v>331</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>575</v>
+        <v>568</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>576</v>
+        <v>569</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>577</v>
+        <v>570</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
@@ -10479,13 +10564,13 @@
         <v>331</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>683</v>
+        <v>676</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>685</v>
+        <v>678</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>684</v>
+        <v>677</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
@@ -10612,16 +10697,16 @@
         <v>330</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>686</v>
+        <v>679</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>475</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>687</v>
+        <v>680</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>688</v>
+        <v>681</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
@@ -10629,7 +10714,7 @@
         <v>1</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>711</v>
+        <v>704</v>
       </c>
       <c r="C52" s="12">
         <v>1</v>
@@ -10638,13 +10723,13 @@
         <v>331</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>712</v>
+        <v>705</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>713</v>
+        <v>706</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>714</v>
+        <v>707</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
@@ -10661,13 +10746,13 @@
         <v>330</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>723</v>
+        <v>716</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>654</v>
+        <v>647</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>724</v>
+        <v>717</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
@@ -10684,13 +10769,13 @@
         <v>330</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>827</v>
+        <v>820</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>828</v>
+        <v>821</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>829</v>
+        <v>822</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
@@ -10698,25 +10783,25 @@
         <v>1</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>841</v>
+        <v>834</v>
       </c>
       <c r="C55" s="12">
         <v>1</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>842</v>
+        <v>835</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>843</v>
+        <v>836</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>844</v>
+        <v>837</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>845</v>
+        <v>838</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>846</v>
+        <v>839</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
@@ -10724,7 +10809,7 @@
         <v>1</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>868</v>
+        <v>861</v>
       </c>
       <c r="C56" s="12">
         <v>1</v>
@@ -10733,29 +10818,69 @@
         <v>202</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>869</v>
+        <v>862</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>202</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>870</v>
+        <v>863</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>871</v>
+        <v>864</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C57" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="C57" s="12">
+        <v>4</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>867</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>868</v>
+      </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C58" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="C58" s="12">
+        <v>4</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="F58" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>867</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>868</v>
+      </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" s="10" t="b">
@@ -11108,27 +11233,45 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>549</v>
+        <v>542</v>
       </c>
       <c r="C4" t="s">
         <v>99</v>
       </c>
       <c r="D4" t="s">
-        <v>548</v>
+        <v>541</v>
       </c>
       <c r="E4" t="s">
         <v>103</v>
       </c>
       <c r="F4" t="s">
-        <v>546</v>
+        <v>539</v>
       </c>
       <c r="G4" t="s">
-        <v>547</v>
+        <v>540</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>883</v>
+      </c>
+      <c r="C5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D5" t="s">
+        <v>884</v>
+      </c>
+      <c r="E5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" t="s">
+        <v>885</v>
+      </c>
+      <c r="G5" t="s">
+        <v>886</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -11225,7 +11368,7 @@
         <v>114</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>619</v>
+        <v>612</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>115</v>
@@ -11251,7 +11394,7 @@
         <v>171</v>
       </c>
       <c r="E2" t="s">
-        <v>671</v>
+        <v>664</v>
       </c>
       <c r="F2" t="s">
         <v>172</v>
@@ -11277,7 +11420,7 @@
         <v>119</v>
       </c>
       <c r="E3" t="s">
-        <v>670</v>
+        <v>663</v>
       </c>
       <c r="F3" t="s">
         <v>120</v>
@@ -11300,7 +11443,7 @@
         <v>171</v>
       </c>
       <c r="E4" t="s">
-        <v>672</v>
+        <v>665</v>
       </c>
       <c r="F4" t="s">
         <v>464</v>
@@ -11320,22 +11463,22 @@
         <v>116</v>
       </c>
       <c r="C5" t="s">
-        <v>666</v>
+        <v>659</v>
       </c>
       <c r="D5" t="s">
         <v>119</v>
       </c>
       <c r="E5" t="s">
-        <v>669</v>
+        <v>662</v>
       </c>
       <c r="F5" t="s">
         <v>469</v>
       </c>
       <c r="G5" t="s">
-        <v>667</v>
+        <v>660</v>
       </c>
       <c r="H5" t="s">
-        <v>668</v>
+        <v>661</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -11349,7 +11492,7 @@
         <v>524</v>
       </c>
       <c r="E6" t="s">
-        <v>618</v>
+        <v>611</v>
       </c>
       <c r="F6" t="s">
         <v>172</v>
@@ -11369,19 +11512,19 @@
         <v>523</v>
       </c>
       <c r="C7" t="s">
-        <v>632</v>
+        <v>625</v>
       </c>
       <c r="E7" t="s">
-        <v>636</v>
+        <v>629</v>
       </c>
       <c r="F7" t="s">
-        <v>634</v>
+        <v>627</v>
       </c>
       <c r="G7" t="s">
-        <v>633</v>
+        <v>626</v>
       </c>
       <c r="H7" t="s">
-        <v>635</v>
+        <v>628</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -11395,7 +11538,7 @@
         <v>468</v>
       </c>
       <c r="E8" t="s">
-        <v>617</v>
+        <v>610</v>
       </c>
       <c r="F8" t="s">
         <v>469</v>
@@ -11424,10 +11567,10 @@
         <v>464</v>
       </c>
       <c r="G9" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="H9" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -11438,19 +11581,19 @@
         <v>467</v>
       </c>
       <c r="C10" t="s">
-        <v>613</v>
+        <v>606</v>
       </c>
       <c r="E10" t="s">
-        <v>617</v>
+        <v>610</v>
       </c>
       <c r="F10" t="s">
-        <v>614</v>
+        <v>607</v>
       </c>
       <c r="G10" t="s">
-        <v>615</v>
+        <v>608</v>
       </c>
       <c r="H10" t="s">
-        <v>616</v>
+        <v>609</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -11461,19 +11604,19 @@
         <v>467</v>
       </c>
       <c r="C11" t="s">
-        <v>629</v>
+        <v>622</v>
       </c>
       <c r="E11" t="s">
-        <v>617</v>
+        <v>610</v>
       </c>
       <c r="F11" t="s">
-        <v>614</v>
+        <v>607</v>
       </c>
       <c r="G11" t="s">
-        <v>630</v>
+        <v>623</v>
       </c>
       <c r="H11" t="s">
-        <v>631</v>
+        <v>624</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -11484,19 +11627,19 @@
         <v>523</v>
       </c>
       <c r="C12" t="s">
-        <v>764</v>
+        <v>757</v>
       </c>
       <c r="E12" t="s">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="F12" t="s">
-        <v>766</v>
+        <v>759</v>
       </c>
       <c r="G12" t="s">
-        <v>767</v>
+        <v>760</v>
       </c>
       <c r="H12" t="s">
-        <v>768</v>
+        <v>761</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -11510,16 +11653,16 @@
         <v>524</v>
       </c>
       <c r="E13" t="s">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="F13" t="s">
-        <v>766</v>
+        <v>759</v>
       </c>
       <c r="G13" t="s">
-        <v>816</v>
+        <v>809</v>
       </c>
       <c r="H13" t="s">
-        <v>817</v>
+        <v>810</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -11600,16 +11743,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>637</v>
+        <v>630</v>
       </c>
       <c r="C2" t="s">
-        <v>646</v>
+        <v>639</v>
       </c>
       <c r="D2" t="s">
-        <v>638</v>
+        <v>631</v>
       </c>
       <c r="E2" t="s">
-        <v>639</v>
+        <v>632</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -11617,16 +11760,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>637</v>
+        <v>630</v>
       </c>
       <c r="C3" t="s">
-        <v>645</v>
+        <v>638</v>
       </c>
       <c r="D3" t="s">
-        <v>647</v>
+        <v>640</v>
       </c>
       <c r="E3" t="s">
-        <v>648</v>
+        <v>641</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -11651,13 +11794,13 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>610</v>
+        <v>603</v>
       </c>
       <c r="D5" t="s">
-        <v>612</v>
+        <v>605</v>
       </c>
       <c r="E5" t="s">
-        <v>611</v>
+        <v>604</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -11682,16 +11825,16 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>673</v>
+        <v>666</v>
       </c>
       <c r="C7" t="s">
-        <v>676</v>
+        <v>669</v>
       </c>
       <c r="D7" t="s">
-        <v>674</v>
+        <v>667</v>
       </c>
       <c r="E7" t="s">
-        <v>675</v>
+        <v>668</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -11713,16 +11856,16 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>707</v>
+        <v>700</v>
       </c>
       <c r="C9" t="s">
-        <v>708</v>
+        <v>701</v>
       </c>
       <c r="D9" t="s">
-        <v>709</v>
+        <v>702</v>
       </c>
       <c r="E9" t="s">
-        <v>710</v>
+        <v>703</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -11730,16 +11873,13 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>540</v>
-      </c>
-      <c r="C10" t="s">
-        <v>541</v>
+        <v>882</v>
       </c>
       <c r="D10" t="s">
-        <v>542</v>
+        <v>880</v>
       </c>
       <c r="E10" t="s">
-        <v>543</v>
+        <v>881</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -11761,16 +11901,16 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>562</v>
+        <v>555</v>
       </c>
       <c r="C12" t="s">
-        <v>563</v>
+        <v>556</v>
       </c>
       <c r="D12" t="s">
-        <v>564</v>
+        <v>557</v>
       </c>
       <c r="E12" t="s">
-        <v>565</v>
+        <v>558</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -11778,16 +11918,16 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>679</v>
+        <v>672</v>
       </c>
       <c r="C13" t="s">
-        <v>680</v>
+        <v>673</v>
       </c>
       <c r="D13" t="s">
-        <v>681</v>
+        <v>674</v>
       </c>
       <c r="E13" t="s">
-        <v>682</v>
+        <v>675</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -11795,16 +11935,16 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>679</v>
+        <v>672</v>
       </c>
       <c r="C14" t="s">
-        <v>689</v>
+        <v>682</v>
       </c>
       <c r="D14" t="s">
-        <v>690</v>
+        <v>683</v>
       </c>
       <c r="E14" t="s">
-        <v>691</v>
+        <v>684</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -11812,16 +11952,16 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>719</v>
+        <v>712</v>
       </c>
       <c r="C15" t="s">
-        <v>720</v>
+        <v>713</v>
       </c>
       <c r="D15" t="s">
-        <v>721</v>
+        <v>714</v>
       </c>
       <c r="E15" t="s">
-        <v>722</v>
+        <v>715</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -11829,16 +11969,16 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>725</v>
+        <v>718</v>
       </c>
       <c r="C16" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
       <c r="D16" t="s">
-        <v>727</v>
+        <v>720</v>
       </c>
       <c r="E16" t="s">
-        <v>728</v>
+        <v>721</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -11846,13 +11986,13 @@
         <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>559</v>
+        <v>552</v>
       </c>
       <c r="D17" t="s">
-        <v>560</v>
+        <v>553</v>
       </c>
       <c r="E17" t="s">
-        <v>561</v>
+        <v>554</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -11860,16 +12000,16 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>744</v>
+        <v>737</v>
       </c>
       <c r="C18" t="s">
-        <v>746</v>
+        <v>739</v>
       </c>
       <c r="D18" t="s">
-        <v>745</v>
+        <v>738</v>
       </c>
       <c r="E18" t="s">
-        <v>747</v>
+        <v>740</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -11911,16 +12051,16 @@
         <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>703</v>
+        <v>696</v>
       </c>
       <c r="C21" t="s">
-        <v>704</v>
+        <v>697</v>
       </c>
       <c r="D21" t="s">
-        <v>706</v>
+        <v>699</v>
       </c>
       <c r="E21" t="s">
-        <v>705</v>
+        <v>698</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -11993,16 +12133,16 @@
         <v>1</v>
       </c>
       <c r="B26" t="s">
+        <v>879</v>
+      </c>
+      <c r="C26" t="s">
         <v>536</v>
       </c>
-      <c r="C26" t="s">
-        <v>538</v>
-      </c>
       <c r="D26" t="s">
-        <v>537</v>
+        <v>877</v>
       </c>
       <c r="E26" t="s">
-        <v>539</v>
+        <v>878</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -12044,13 +12184,13 @@
         <v>1</v>
       </c>
       <c r="B29" t="s">
-        <v>749</v>
+        <v>742</v>
       </c>
       <c r="D29" t="s">
-        <v>748</v>
+        <v>741</v>
       </c>
       <c r="E29" t="s">
-        <v>750</v>
+        <v>743</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
@@ -12058,16 +12198,16 @@
         <v>0</v>
       </c>
       <c r="B30" t="s">
-        <v>752</v>
+        <v>745</v>
       </c>
       <c r="C30" t="s">
-        <v>753</v>
+        <v>746</v>
       </c>
       <c r="D30" t="s">
-        <v>751</v>
+        <v>744</v>
       </c>
       <c r="E30" t="s">
-        <v>757</v>
+        <v>750</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
@@ -12075,16 +12215,16 @@
         <v>0</v>
       </c>
       <c r="B31" t="s">
-        <v>755</v>
+        <v>748</v>
       </c>
       <c r="C31" t="s">
-        <v>753</v>
+        <v>746</v>
       </c>
       <c r="D31" t="s">
-        <v>754</v>
+        <v>747</v>
       </c>
       <c r="E31" t="s">
-        <v>756</v>
+        <v>749</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
@@ -12092,16 +12232,16 @@
         <v>0</v>
       </c>
       <c r="B32" t="s">
-        <v>760</v>
+        <v>753</v>
       </c>
       <c r="C32" t="s">
         <v>218</v>
       </c>
       <c r="D32" t="s">
-        <v>758</v>
+        <v>751</v>
       </c>
       <c r="E32" t="s">
-        <v>759</v>
+        <v>752</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
@@ -12109,16 +12249,16 @@
         <v>1</v>
       </c>
       <c r="B33" t="s">
-        <v>562</v>
+        <v>555</v>
       </c>
       <c r="C33" t="s">
-        <v>762</v>
+        <v>755</v>
       </c>
       <c r="D33" t="s">
-        <v>761</v>
+        <v>754</v>
       </c>
       <c r="E33" t="s">
-        <v>763</v>
+        <v>756</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
@@ -12234,7 +12374,7 @@
         <v>197</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>243</v>
+        <v>888</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>246</v>
@@ -12359,16 +12499,16 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>824</v>
+        <v>817</v>
       </c>
       <c r="C8" t="s">
-        <v>825</v>
+        <v>818</v>
       </c>
       <c r="D8" t="s">
-        <v>826</v>
+        <v>819</v>
       </c>
       <c r="F8" t="s">
-        <v>823</v>
+        <v>816</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -12376,13 +12516,13 @@
         <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>832</v>
+        <v>825</v>
       </c>
       <c r="C9" t="s">
-        <v>831</v>
+        <v>824</v>
       </c>
       <c r="D9" t="s">
-        <v>830</v>
+        <v>823</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -12390,21 +12530,36 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>837</v>
+        <v>830</v>
       </c>
       <c r="C10" t="s">
-        <v>838</v>
+        <v>831</v>
       </c>
       <c r="D10" t="s">
-        <v>840</v>
+        <v>833</v>
       </c>
       <c r="E10" t="s">
-        <v>839</v>
+        <v>832</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>889</v>
+      </c>
+      <c r="C11" t="s">
+        <v>887</v>
+      </c>
+      <c r="D11" t="s">
+        <v>890</v>
+      </c>
+      <c r="E11" t="s">
+        <v>887</v>
+      </c>
+      <c r="F11" t="s">
+        <v>891</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
fixed RP2350A reference design
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FB77531-BB17-43DB-8EB8-BF3D267EFD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D612E23B-E267-4084-936D-D6440F7D8B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="11170" firstSheet="1" activeTab="6" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="3040" yWindow="3040" windowWidth="19200" windowHeight="11170" firstSheet="1" activeTab="6" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1527" uniqueCount="892">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1540" uniqueCount="901">
   <si>
     <t>Capacitance</t>
   </si>
@@ -2735,6 +2735,33 @@
   </si>
   <si>
     <t>https://www.winson.com.tw/uploads/images/WCS1600.pdf</t>
+  </si>
+  <si>
+    <t>Bridge (UART-RS485)</t>
+  </si>
+  <si>
+    <t>THVD1400DR</t>
+  </si>
+  <si>
+    <t>1/1 Transceiver Half RS422, RS485 8-SOIC</t>
+  </si>
+  <si>
+    <t>7,12V</t>
+  </si>
+  <si>
+    <t>400W</t>
+  </si>
+  <si>
+    <t>CDSOT23-SM712</t>
+  </si>
+  <si>
+    <t>26V, 14V Clamp 17A (8/20µs) Ipp Tvs Diode Surface Mount SOT-23-3</t>
+  </si>
+  <si>
+    <t>Tube</t>
+  </si>
+  <si>
+    <t>2mL Tube</t>
   </si>
 </sst>
 </file>
@@ -3151,23 +3178,6 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
@@ -3237,6 +3247,23 @@
         </ext>
       </extLst>
     </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="1"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3281,13 +3308,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I49" totalsRowShown="0">
   <autoFilter ref="A1:I49" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="78"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="75"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="77"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="74"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="76"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="75"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="72"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -3482,20 +3509,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="71">
   <autoFilter ref="A1:H100" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H100">
     <sortCondition ref="B1:B100"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="73"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="72"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="71"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="70"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="69"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="68"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="67"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="66"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3518,13 +3545,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="62">
   <autoFilter ref="A1:H20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H20">
     <sortCondition ref="B1:B20"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="64"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="61"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -3544,8 +3571,8 @@
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="63"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="60"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="59"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -3555,11 +3582,11 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="78">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series / Purpose" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="77"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series / Purpose" dataDxfId="76"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -11667,7 +11694,25 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B14" t="s">
+        <v>523</v>
+      </c>
+      <c r="C14" t="s">
+        <v>895</v>
+      </c>
+      <c r="E14" t="s">
+        <v>896</v>
+      </c>
+      <c r="F14" t="s">
+        <v>846</v>
+      </c>
+      <c r="G14" t="s">
+        <v>897</v>
+      </c>
+      <c r="H14" t="s">
+        <v>898</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -12263,7 +12308,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B34" t="s">
+        <v>892</v>
+      </c>
+      <c r="D34" t="s">
+        <v>893</v>
+      </c>
+      <c r="E34" t="s">
+        <v>894</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
@@ -12564,7 +12618,19 @@
     </row>
     <row r="12" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B12" t="s">
+        <v>899</v>
+      </c>
+      <c r="C12" t="s">
+        <v>900</v>
+      </c>
+      <c r="D12" t="s">
+        <v>900</v>
+      </c>
+      <c r="E12" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>